<commit_message>
Published state of ETDataset for deploy 2026-09
</commit_message>
<xml_diff>
--- a/analyses/6_residences_analysis.xlsx
+++ b/analyses/6_residences_analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathijsbijkerk/Github/etdataset/analyses/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathijsbijkerk/Github/etm-ecosystem/etdataset/analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{177A9909-FF8D-5D4E-BA8D-A632A8C7BE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47113DC-6C3D-7E43-ABF3-404E7C3BD957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15600" yWindow="-33340" windowWidth="30080" windowHeight="16200" tabRatio="932" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11300" yWindow="-28200" windowWidth="51200" windowHeight="27300" tabRatio="932" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Sheet" sheetId="34" r:id="rId1"/>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="934">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="933">
   <si>
     <t>Changelog</t>
   </si>
@@ -2121,9 +2121,6 @@
     <t>households_space_heater_heatpump_ground_water_electricity.converter</t>
   </si>
   <si>
-    <t>households_space_heater_heatpump_air_water_electricity.converter</t>
-  </si>
-  <si>
     <t>households_space_heater_wood_pellets.converter</t>
   </si>
   <si>
@@ -2145,9 +2142,6 @@
     <t>households_water_heater_heatpump_ground_water_electricity.converter</t>
   </si>
   <si>
-    <t>households_water_heater_heatpump_air_water_electricity.converter</t>
-  </si>
-  <si>
     <t>households_water_heater_wood_pellets.converter</t>
   </si>
   <si>
@@ -2215,9 +2209,6 @@
   </si>
   <si>
     <t>Extract data from Etsource</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Here, the technological specifications are imported from Etsource (automatically). These values are not country-specific and cannot be changed. </t>
   </si>
   <si>
     <t>cleaned up fuel aggregation sheet and tech_specs sheet</t>
@@ -2368,9 +2359,6 @@
     <t>electricity-driven heat pump (air)</t>
   </si>
   <si>
-    <t>households_space_heater_hybrid_heatpump_air_water_electricity.converter</t>
-  </si>
-  <si>
     <t>households_space_heater_hybrid_heatpump_air_water_electricity</t>
   </si>
   <si>
@@ -2416,9 +2404,6 @@
     <t>Hybrid heatpump, gas part (hot water)</t>
   </si>
   <si>
-    <t>households_water_heater_hybrid_heatpump_air_water_electricity.converter</t>
-  </si>
-  <si>
     <t>Eff_space_heating_hhp_gas</t>
   </si>
   <si>
@@ -2933,6 +2918,18 @@
   </si>
   <si>
     <t>Add surface water technologies to export CSVs with zero share.</t>
+  </si>
+  <si>
+    <t>August 19, 2026</t>
+  </si>
+  <si>
+    <t>August 19, 2025</t>
+  </si>
+  <si>
+    <t>The hardcoded specs for HHPs in the 'technical_specs' sheet were outdated and too high for the space heating part. These have been updated based the new node source analyses for the corresponding technology. Additionally, for the hot water part, we assume that the cutoff COP is set at 6.0, effectively ensuring that only network gas is used. To reflect this, the input of network gas is set to 100% and electricity to 0%. These are improvements of the fix in 2.21.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Here, the technological specifications are imported from ETSource (automatically). These values are not country-specific and cannot be changed. </t>
   </si>
 </sst>
 </file>
@@ -6649,7 +6646,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="606">
+  <cellXfs count="607">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -7658,13 +7655,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
@@ -7691,7 +7690,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2404">
     <cellStyle name="Calculation" xfId="1524" builtinId="22" customBuiltin="1"/>
@@ -13612,6 +13610,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Cover sheet"/>
       <sheetName val="Dashboard"/>
@@ -13987,7 +13988,7 @@
       </c>
       <c r="C5" s="365">
         <f>MAX(Changelog!D:D)</f>
-        <v>2.25</v>
+        <v>2.2599999999999998</v>
       </c>
       <c r="D5" s="7"/>
     </row>
@@ -13996,7 +13997,7 @@
         <v>306</v>
       </c>
       <c r="C6" s="133" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="D6" s="7"/>
     </row>
@@ -14014,7 +14015,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="335" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="D8" s="7"/>
     </row>
@@ -14023,7 +14024,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="D9" s="7"/>
     </row>
@@ -14032,7 +14033,7 @@
         <v>18</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="D10" s="10"/>
     </row>
@@ -14243,12 +14244,12 @@
       <c r="E4" s="5"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>379</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="596"/>
-      <c r="E5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="597"/>
+      <c r="E5" s="598"/>
       <c r="F5" s="143"/>
     </row>
     <row r="6" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -14656,13 +14657,13 @@
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>514</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="596"/>
-      <c r="E5" s="596"/>
-      <c r="F5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="597"/>
+      <c r="E5" s="597"/>
+      <c r="F5" s="598"/>
       <c r="G5" s="144"/>
     </row>
     <row r="6" spans="2:7" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -15353,14 +15354,14 @@
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>278</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="596"/>
-      <c r="E5" s="596"/>
-      <c r="F5" s="596"/>
-      <c r="G5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="597"/>
+      <c r="E5" s="597"/>
+      <c r="F5" s="597"/>
+      <c r="G5" s="598"/>
     </row>
     <row r="6" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:18" x14ac:dyDescent="0.2">
@@ -15377,7 +15378,7 @@
       <c r="J7" s="49"/>
       <c r="K7" s="27"/>
       <c r="M7" s="534" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="N7" s="536"/>
       <c r="O7" s="536"/>
@@ -15427,22 +15428,22 @@
         <v>645</v>
       </c>
       <c r="M9" s="538" t="s">
-        <v>780</v>
+        <v>775</v>
       </c>
       <c r="N9" s="539" t="s">
-        <v>779</v>
+        <v>774</v>
       </c>
       <c r="O9" s="539" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
       <c r="P9" s="527" t="s">
         <v>659</v>
       </c>
       <c r="Q9" s="527" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="R9" s="535" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.2">
@@ -15810,7 +15811,7 @@
     <row r="24" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B24" s="46"/>
       <c r="C24" s="220" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="D24" s="507" t="e">
         <f>'Technology split final demand'!I20</f>
@@ -15828,7 +15829,7 @@
       <c r="K24" s="253"/>
       <c r="M24" s="540">
         <f>technical_specs!O20</f>
-        <v>4.4999999999999885</v>
+        <v>3.5000066339098939</v>
       </c>
       <c r="N24" s="527" t="e">
         <f>F24*M24</f>
@@ -15854,7 +15855,7 @@
     <row r="25" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B25" s="46"/>
       <c r="C25" s="221" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="D25" s="504" t="e">
         <f>'Technology split final demand'!I21</f>
@@ -15880,7 +15881,7 @@
     <row r="26" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B26" s="222"/>
       <c r="C26" s="506" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="D26" s="141"/>
       <c r="E26" s="238"/>
@@ -16183,7 +16184,7 @@
       <c r="K37" s="253"/>
       <c r="M37" s="540">
         <f>technical_specs!O33</f>
-        <v>3.0000000000000044</v>
+        <v>1</v>
       </c>
       <c r="N37" s="527" t="e">
         <f>F37*M37</f>
@@ -17022,13 +17023,13 @@
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="2:10" s="67" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>228</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="596"/>
-      <c r="E5" s="596"/>
-      <c r="F5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="597"/>
+      <c r="E5" s="597"/>
+      <c r="F5" s="598"/>
       <c r="G5" s="143"/>
     </row>
     <row r="6" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -17061,7 +17062,7 @@
         <v>435</v>
       </c>
       <c r="E9" s="73" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="F9" s="73" t="s">
         <v>479</v>
@@ -17379,7 +17380,7 @@
       </c>
       <c r="F20" s="460">
         <f>Eff_space_heating_hhp_heatpump</f>
-        <v>4.4999999999999885</v>
+        <v>3.5000066339098939</v>
       </c>
       <c r="G20" s="172">
         <v>1</v>
@@ -17734,20 +17735,20 @@
         <f>Dashboard!E53</f>
         <v>0</v>
       </c>
-      <c r="E33" s="165">
+      <c r="E33" s="165" t="e">
         <f>D33*(1-technical_specs!Q34)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F33" s="460">
         <f>Eff_hot_water_hhp_heatpump</f>
-        <v>3.0000000000000044</v>
+        <v>1</v>
       </c>
       <c r="G33" s="172">
         <v>1</v>
       </c>
-      <c r="H33" s="248">
+      <c r="H33" s="248" t="e">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="I33" s="505" t="e">
         <f t="shared" si="3"/>
@@ -17762,9 +17763,9 @@
         <v>Hybrid heatpump, gas part (hot water)</v>
       </c>
       <c r="D34" s="165"/>
-      <c r="E34" s="165">
+      <c r="E34" s="165" t="e">
         <f>D33*technical_specs!Q34</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F34" s="460">
         <f>Eff_hot_water_hhp_gas</f>
@@ -18387,14 +18388,14 @@
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="2:13" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>227</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="596"/>
-      <c r="E5" s="596"/>
-      <c r="F5" s="596"/>
-      <c r="G5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="597"/>
+      <c r="E5" s="597"/>
+      <c r="F5" s="597"/>
+      <c r="G5" s="598"/>
     </row>
     <row r="6" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:13" x14ac:dyDescent="0.2">
@@ -18457,7 +18458,7 @@
         <v>527</v>
       </c>
       <c r="L9" s="103" t="s">
-        <v>836</v>
+        <v>831</v>
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.2">
@@ -18620,10 +18621,10 @@
     <row r="24" spans="2:12" ht="78" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="377"/>
       <c r="C24" s="377"/>
-      <c r="K24" s="601" t="s">
-        <v>837</v>
-      </c>
-      <c r="L24" s="602"/>
+      <c r="K24" s="603" t="s">
+        <v>832</v>
+      </c>
+      <c r="L24" s="604"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B25" s="377"/>
@@ -18688,19 +18689,19 @@
   <sheetData>
     <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="112" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="603" t="s">
-        <v>792</v>
-      </c>
-      <c r="C4" s="604"/>
+      <c r="B4" s="605" t="s">
+        <v>787</v>
+      </c>
+      <c r="C4" s="606"/>
       <c r="D4" s="17"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B5" s="594"/>
-      <c r="C5" s="596"/>
+      <c r="B5" s="596"/>
+      <c r="C5" s="597"/>
       <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -18734,22 +18735,22 @@
       <c r="B8" s="546"/>
       <c r="C8" s="547"/>
       <c r="D8" s="548" t="s">
+        <v>791</v>
+      </c>
+      <c r="E8" s="549" t="s">
+        <v>792</v>
+      </c>
+      <c r="F8" s="548" t="s">
+        <v>794</v>
+      </c>
+      <c r="G8" s="548" t="s">
+        <v>775</v>
+      </c>
+      <c r="H8" s="549" t="s">
         <v>796</v>
       </c>
-      <c r="E8" s="549" t="s">
+      <c r="I8" s="550" t="s">
         <v>797</v>
-      </c>
-      <c r="F8" s="548" t="s">
-        <v>799</v>
-      </c>
-      <c r="G8" s="548" t="s">
-        <v>780</v>
-      </c>
-      <c r="H8" s="549" t="s">
-        <v>801</v>
-      </c>
-      <c r="I8" s="550" t="s">
-        <v>802</v>
       </c>
       <c r="J8" s="56"/>
       <c r="K8" s="56"/>
@@ -18757,7 +18758,7 @@
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="56"/>
       <c r="B9" s="545" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="C9" s="96" t="s">
         <v>384</v>
@@ -18806,7 +18807,7 @@
       </c>
       <c r="G10" s="451">
         <f>technical_specs!O20</f>
-        <v>4.4999999999999885</v>
+        <v>3.5000066339098939</v>
       </c>
       <c r="H10" s="1" t="e">
         <f>D10*E10*F10</f>
@@ -18823,7 +18824,7 @@
       <c r="A11" s="56"/>
       <c r="B11" s="545"/>
       <c r="C11" s="56" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="D11" s="56"/>
       <c r="E11" s="56"/>
@@ -18859,17 +18860,17 @@
       <c r="C13" s="547"/>
       <c r="D13" s="547"/>
       <c r="E13" s="549" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="F13" s="549" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="G13" s="549"/>
       <c r="H13" s="549" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="I13" s="550" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="J13" s="56"/>
       <c r="K13" s="56"/>
@@ -18877,7 +18878,7 @@
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="56"/>
       <c r="B14" s="453" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="C14" s="56" t="s">
         <v>384</v>
@@ -18925,7 +18926,7 @@
       </c>
       <c r="G15" s="551">
         <f>technical_specs!O33</f>
-        <v>3.0000000000000044</v>
+        <v>1</v>
       </c>
       <c r="H15" s="1" t="e">
         <f>D15*E15*F15</f>
@@ -18941,7 +18942,7 @@
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B16" s="28"/>
       <c r="C16" s="56" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="D16" s="451"/>
       <c r="E16" s="451"/>
@@ -19161,11 +19162,11 @@
       <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:14" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>484</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="598"/>
     </row>
     <row r="6" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="56"/>
@@ -19218,7 +19219,7 @@
         <v>214</v>
       </c>
       <c r="G9" s="180" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="H9" s="180" t="s">
         <v>586</v>
@@ -19567,7 +19568,7 @@
       </c>
       <c r="F20" s="200">
         <f>technical_specs!R20</f>
-        <v>4.4999999999999885</v>
+        <v>3.5000066339098939</v>
       </c>
       <c r="G20" s="511" t="e">
         <f t="shared" si="2"/>
@@ -19995,7 +19996,7 @@
       </c>
       <c r="F33" s="200">
         <f>technical_specs!R33</f>
-        <v>3.0000000000000044</v>
+        <v>1</v>
       </c>
       <c r="G33" s="511" t="e">
         <f t="shared" si="7"/>
@@ -21127,7 +21128,7 @@
         <v>41535</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="D26" s="24">
         <v>2.09</v>
@@ -21138,7 +21139,7 @@
         <v>41535</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="D27" s="24">
         <v>2.1</v>
@@ -21149,7 +21150,7 @@
         <v>41561</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="D28" s="15">
         <v>2.11</v>
@@ -21160,7 +21161,7 @@
         <v>41562</v>
       </c>
       <c r="C29" s="556" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="D29" s="15">
         <v>2.12</v>
@@ -21171,7 +21172,7 @@
         <v>41578</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="D30" s="15">
         <v>2.13</v>
@@ -21182,7 +21183,7 @@
         <v>41618</v>
       </c>
       <c r="C31" s="37" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="D31" s="15">
         <v>2.14</v>
@@ -21190,10 +21191,10 @@
     </row>
     <row r="32" spans="2:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B32" s="334" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="C32" s="37" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="D32" s="15">
         <v>2.15</v>
@@ -21201,10 +21202,10 @@
     </row>
     <row r="33" spans="2:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B33" s="334" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="C33" s="37" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="D33" s="15">
         <v>2.16</v>
@@ -21212,10 +21213,10 @@
     </row>
     <row r="34" spans="2:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B34" s="334" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="D34" s="15">
         <v>2.17</v>
@@ -21223,10 +21224,10 @@
     </row>
     <row r="35" spans="2:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
-        <v>767</v>
+        <v>762</v>
       </c>
       <c r="C35" s="37" t="s">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="D35" s="15">
         <v>2.1800000000000002</v>
@@ -21234,10 +21235,10 @@
     </row>
     <row r="36" spans="2:4" ht="51" x14ac:dyDescent="0.2">
       <c r="B36" s="16" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
       <c r="C36" s="557" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="D36" s="15">
         <v>2.19</v>
@@ -21245,10 +21246,10 @@
     </row>
     <row r="37" spans="2:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B37" s="334" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
       <c r="C37" s="37" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
       <c r="D37" s="15">
         <v>2.2000000000000002</v>
@@ -21256,10 +21257,10 @@
     </row>
     <row r="38" spans="2:4" ht="85" x14ac:dyDescent="0.2">
       <c r="B38" s="334" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="C38" s="37" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="D38" s="15">
         <v>2.21</v>
@@ -21267,10 +21268,10 @@
     </row>
     <row r="39" spans="2:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B39" s="334" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="C39" s="37" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="D39" s="15">
         <v>2.2200000000000002</v>
@@ -21278,10 +21279,10 @@
     </row>
     <row r="40" spans="2:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B40" s="334" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="D40" s="15">
         <v>2.23</v>
@@ -21289,10 +21290,10 @@
     </row>
     <row r="41" spans="2:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B41" s="334" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="C41" s="37" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="D41" s="15">
         <v>2.2400000000000002</v>
@@ -21300,19 +21301,25 @@
     </row>
     <row r="42" spans="2:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B42" s="334" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
       <c r="C42" s="37" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
       <c r="D42" s="15">
         <v>2.25</v>
       </c>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B43" s="334"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="15"/>
+    <row r="43" spans="2:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="B43" s="334" t="s">
+        <v>929</v>
+      </c>
+      <c r="C43" s="37" t="s">
+        <v>931</v>
+      </c>
+      <c r="D43" s="15">
+        <v>2.2599999999999998</v>
+      </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B44" s="334"/>
@@ -21579,9 +21586,9 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>929</v>
-      </c>
-      <c r="B6" s="605">
+        <v>924</v>
+      </c>
+      <c r="B6" s="594">
         <v>0</v>
       </c>
     </row>
@@ -21636,7 +21643,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="B5" s="171" t="e">
         <f>'Technology Shares'!F11</f>
@@ -21703,7 +21710,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="B6" s="171" t="e">
         <f>'Technology Shares'!F16</f>
@@ -21712,9 +21719,9 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>930</v>
-      </c>
-      <c r="B7" s="605">
+        <v>925</v>
+      </c>
+      <c r="B7" s="594">
         <v>0</v>
       </c>
     </row>
@@ -21770,7 +21777,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="B5" s="171" t="e">
         <f>'Technology Shares'!F21</f>
@@ -21837,7 +21844,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="B6" s="171" t="e">
         <f>'Technology Shares'!F26</f>
@@ -21846,9 +21853,9 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>931</v>
-      </c>
-      <c r="B7" s="605">
+        <v>926</v>
+      </c>
+      <c r="B7" s="594">
         <v>0</v>
       </c>
     </row>
@@ -22271,20 +22278,20 @@
     </row>
     <row r="39" spans="2:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="405" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="C39" s="406"/>
     </row>
     <row r="40" spans="2:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="405" t="s">
-        <v>832</v>
+        <v>827</v>
       </c>
       <c r="C40" s="396"/>
       <c r="D40" s="17"/>
     </row>
     <row r="41" spans="2:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="405" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="C41" s="396"/>
     </row>
@@ -22422,7 +22429,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -22430,12 +22437,12 @@
         <v>481</v>
       </c>
       <c r="B2" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="B3" s="593">
         <f>Dashboard!E87</f>
@@ -22444,7 +22451,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="B4">
         <f>Dashboard!E90</f>
@@ -22453,7 +22460,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="B5">
         <f>Dashboard!E91</f>
@@ -22462,7 +22469,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="B6">
         <f>Dashboard!E92</f>
@@ -22471,7 +22478,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="B7">
         <f>Dashboard!E93</f>
@@ -22480,7 +22487,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="B8">
         <f>Dashboard!E94</f>
@@ -22489,7 +22496,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="B9">
         <f>Dashboard!E95</f>
@@ -22498,7 +22505,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="B10">
         <f>Dashboard!E96</f>
@@ -22507,7 +22514,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="B11">
         <f>Dashboard!E97</f>
@@ -22516,7 +22523,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="B12">
         <f>Dashboard!E98</f>
@@ -22525,7 +22532,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="B13">
         <f>Dashboard!E99</f>
@@ -22534,7 +22541,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="B14">
         <f>Dashboard!E100</f>
@@ -22543,7 +22550,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>897</v>
+        <v>892</v>
       </c>
       <c r="B15">
         <f>Dashboard!E101</f>
@@ -22552,7 +22559,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
       <c r="B16">
         <f>Dashboard!E102</f>
@@ -22561,7 +22568,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>899</v>
+        <v>894</v>
       </c>
       <c r="B17">
         <f>Dashboard!E103</f>
@@ -22570,7 +22577,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
       <c r="B18">
         <f>Dashboard!E104</f>
@@ -22579,7 +22586,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="B19">
         <f>Dashboard!E105</f>
@@ -22588,7 +22595,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
       <c r="B20">
         <f>Dashboard!E106</f>
@@ -22597,7 +22604,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="B21">
         <f>Dashboard!E107</f>
@@ -22606,7 +22613,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="B22">
         <f>Dashboard!E108</f>
@@ -22615,7 +22622,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="B23">
         <f>Dashboard!E109</f>
@@ -22624,7 +22631,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="B24">
         <f>Dashboard!E113</f>
@@ -22633,7 +22640,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="B25">
         <f>Dashboard!E114</f>
@@ -22642,7 +22649,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="B26">
         <f>Dashboard!E115</f>
@@ -22651,7 +22658,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
       <c r="B27">
         <f>Dashboard!E116</f>
@@ -22660,7 +22667,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="B28">
         <f>Dashboard!E117</f>
@@ -22669,7 +22676,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="B29">
         <f>Dashboard!E118</f>
@@ -22678,7 +22685,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="B30">
         <f>Dashboard!E119</f>
@@ -22687,7 +22694,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="B31">
         <f>Dashboard!E120</f>
@@ -22696,7 +22703,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="B32">
         <f>Dashboard!E121</f>
@@ -22705,7 +22712,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="B33">
         <f>Dashboard!E122</f>
@@ -22714,7 +22721,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="B34">
         <f>Dashboard!E123</f>
@@ -22723,7 +22730,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="B35">
         <f>Dashboard!E124</f>
@@ -22732,7 +22739,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="B36">
         <f>Dashboard!E125</f>
@@ -22741,7 +22748,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="B37">
         <f>Dashboard!E126</f>
@@ -22750,7 +22757,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="B38">
         <f>Dashboard!E127</f>
@@ -22759,7 +22766,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="B39">
         <f>Dashboard!E128</f>
@@ -22768,7 +22775,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="B40">
         <f>Dashboard!E129</f>
@@ -22777,7 +22784,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="B41">
         <f>Dashboard!E130</f>
@@ -22786,7 +22793,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="B42">
         <f>Dashboard!E131</f>
@@ -22795,7 +22802,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="B43">
         <f>Dashboard!E132</f>
@@ -22822,7 +22829,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -22835,7 +22842,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="B3">
         <f>IFERROR('HHP input shares'!I9,0.187)</f>
@@ -22853,7 +22860,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="B5">
         <f>1-B4-B3</f>
@@ -22878,7 +22885,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -22891,7 +22898,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="B3">
         <f>IFERROR('HHP input shares'!I14,0.33)</f>
@@ -22909,7 +22916,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="B5">
         <f>1-B4-B3</f>
@@ -22949,7 +22956,7 @@
     </row>
     <row r="6" spans="2:2" ht="102" x14ac:dyDescent="0.2">
       <c r="B6" s="77" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
@@ -23443,10 +23450,10 @@
       <c r="C4" s="5"/>
     </row>
     <row r="5" spans="2:4" ht="79" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>189</v>
       </c>
-      <c r="C5" s="595"/>
+      <c r="C5" s="598"/>
     </row>
     <row r="6" spans="2:4" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
@@ -23596,10 +23603,10 @@
     <row r="28" spans="2:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="36"/>
       <c r="C28" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -24675,7 +24682,7 @@
     </row>
     <row r="182" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B182" s="46" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="C182" s="40" t="s">
         <v>103</v>
@@ -24756,12 +24763,12 @@
       <c r="L4" s="7"/>
     </row>
     <row r="5" spans="2:16" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="594" t="s">
+      <c r="B5" s="596" t="s">
         <v>226</v>
       </c>
-      <c r="C5" s="596"/>
-      <c r="D5" s="596"/>
-      <c r="E5" s="595"/>
+      <c r="C5" s="597"/>
+      <c r="D5" s="597"/>
+      <c r="E5" s="598"/>
       <c r="F5" s="143"/>
       <c r="I5" s="369"/>
       <c r="J5" s="9"/>
@@ -24829,7 +24836,7 @@
       </c>
       <c r="N9" s="13"/>
       <c r="O9" s="375" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="P9" s="376" t="s">
         <v>615</v>
@@ -24866,7 +24873,7 @@
       </c>
       <c r="D11" s="353"/>
       <c r="E11" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="20" t="s">
@@ -25002,10 +25009,10 @@
       <c r="G17" s="344"/>
       <c r="H17" s="585"/>
       <c r="I17" t="s">
-        <v>885</v>
-      </c>
-      <c r="K17" s="597" t="s">
-        <v>882</v>
+        <v>880</v>
+      </c>
+      <c r="K17" s="599" t="s">
+        <v>877</v>
       </c>
       <c r="L17" s="285"/>
       <c r="M17" s="130"/>
@@ -25020,7 +25027,7 @@
       <c r="F18" s="216"/>
       <c r="G18" s="343"/>
       <c r="H18" s="586"/>
-      <c r="K18" s="597"/>
+      <c r="K18" s="599"/>
       <c r="L18" s="339"/>
       <c r="M18" s="130"/>
       <c r="N18" s="67"/>
@@ -25030,7 +25037,7 @@
     <row r="19" spans="2:16" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B19" s="35"/>
       <c r="C19" s="581" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="D19" s="324"/>
       <c r="E19" s="216"/>
@@ -25108,7 +25115,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="292" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="N21" s="67"/>
       <c r="O21" s="368" t="s">
@@ -25257,7 +25264,7 @@
     <row r="27" spans="2:16" ht="17" x14ac:dyDescent="0.2">
       <c r="B27" s="35"/>
       <c r="C27" s="1" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="D27" s="324" t="s">
         <v>213</v>
@@ -25331,7 +25338,7 @@
     <row r="30" spans="2:16" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B30" s="35"/>
       <c r="C30" s="581" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="D30" s="324"/>
       <c r="E30" s="208"/>
@@ -25348,7 +25355,7 @@
     <row r="31" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B31" s="35"/>
       <c r="C31" s="587" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="D31" s="327"/>
       <c r="E31" s="322"/>
@@ -25368,7 +25375,7 @@
     <row r="32" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B32" s="35"/>
       <c r="C32" s="587" t="s">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="D32" s="327"/>
       <c r="E32" s="322"/>
@@ -25388,7 +25395,7 @@
     <row r="33" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B33" s="35"/>
       <c r="C33" s="587" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="D33" s="327"/>
       <c r="E33" s="322"/>
@@ -25408,7 +25415,7 @@
     <row r="34" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="35"/>
       <c r="C34" s="587" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="D34" s="327"/>
       <c r="E34" s="322"/>
@@ -25428,7 +25435,7 @@
     <row r="35" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B35" s="35"/>
       <c r="C35" s="587" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="D35" s="327"/>
       <c r="E35" s="322"/>
@@ -25448,7 +25455,7 @@
     <row r="36" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B36" s="35"/>
       <c r="C36" s="587" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="D36" s="327"/>
       <c r="E36" s="322"/>
@@ -25468,7 +25475,7 @@
     <row r="37" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B37" s="35"/>
       <c r="C37" s="587" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="D37" s="327"/>
       <c r="E37" s="322"/>
@@ -25488,7 +25495,7 @@
     <row r="38" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B38" s="35"/>
       <c r="C38" s="587" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="D38" s="327"/>
       <c r="E38" s="322"/>
@@ -25508,7 +25515,7 @@
     <row r="39" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B39" s="35"/>
       <c r="C39" s="587" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="D39" s="327"/>
       <c r="E39" s="322"/>
@@ -25527,7 +25534,7 @@
     <row r="40" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B40" s="35"/>
       <c r="C40" s="587" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="D40" s="327"/>
       <c r="E40" s="322"/>
@@ -25540,7 +25547,7 @@
       <c r="M40" s="130"/>
       <c r="N40" s="67"/>
       <c r="O40" s="373" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="P40" s="370"/>
     </row>
@@ -25591,7 +25598,7 @@
     <row r="43" spans="2:16" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B43" s="35"/>
       <c r="C43" s="581" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="D43" s="324"/>
       <c r="E43" s="210"/>
@@ -25608,7 +25615,7 @@
     <row r="44" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B44" s="35"/>
       <c r="C44" s="587" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="D44" s="327"/>
       <c r="E44" s="322"/>
@@ -25628,7 +25635,7 @@
     <row r="45" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B45" s="35"/>
       <c r="C45" s="587" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="D45" s="327"/>
       <c r="E45" s="322"/>
@@ -25648,7 +25655,7 @@
     <row r="46" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B46" s="35"/>
       <c r="C46" s="587" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="D46" s="327"/>
       <c r="E46" s="322"/>
@@ -25668,7 +25675,7 @@
     <row r="47" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B47" s="35"/>
       <c r="C47" s="587" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="D47" s="327"/>
       <c r="E47" s="322"/>
@@ -25688,7 +25695,7 @@
     <row r="48" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B48" s="35"/>
       <c r="C48" s="587" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="D48" s="327"/>
       <c r="E48" s="322"/>
@@ -25708,7 +25715,7 @@
     <row r="49" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B49" s="35"/>
       <c r="C49" s="587" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="D49" s="327"/>
       <c r="E49" s="322"/>
@@ -25728,7 +25735,7 @@
     <row r="50" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B50" s="35"/>
       <c r="C50" s="587" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="D50" s="327"/>
       <c r="E50" s="322"/>
@@ -25748,7 +25755,7 @@
     <row r="51" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B51" s="35"/>
       <c r="C51" s="587" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="D51" s="327"/>
       <c r="E51" s="322"/>
@@ -25768,7 +25775,7 @@
     <row r="52" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B52" s="35"/>
       <c r="C52" s="587" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="D52" s="327"/>
       <c r="E52" s="322"/>
@@ -25788,7 +25795,7 @@
     <row r="53" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B53" s="35"/>
       <c r="C53" s="587" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="D53" s="327"/>
       <c r="E53" s="322"/>
@@ -25801,7 +25808,7 @@
       <c r="M53" s="130"/>
       <c r="N53" s="67"/>
       <c r="O53" s="373" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="P53" s="370"/>
     </row>
@@ -25853,7 +25860,7 @@
     <row r="56" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B56" s="35"/>
       <c r="C56" s="581" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="D56" s="328"/>
       <c r="E56" s="501"/>
@@ -25870,7 +25877,7 @@
     <row r="57" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B57" s="35"/>
       <c r="C57" s="587" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="D57" s="329"/>
       <c r="E57" s="323"/>
@@ -25890,7 +25897,7 @@
     <row r="58" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B58" s="35"/>
       <c r="C58" s="587" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="D58" s="329"/>
       <c r="E58" s="323"/>
@@ -25910,7 +25917,7 @@
     <row r="59" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B59" s="35"/>
       <c r="C59" s="587" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="D59" s="330"/>
       <c r="E59" s="323"/>
@@ -25974,7 +25981,7 @@
     <row r="62" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B62" s="35"/>
       <c r="C62" s="581" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="D62" s="324"/>
       <c r="E62" s="501"/>
@@ -25991,7 +25998,7 @@
     <row r="63" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B63" s="35"/>
       <c r="C63" s="587" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="D63" s="329"/>
       <c r="E63" s="323"/>
@@ -26011,7 +26018,7 @@
     <row r="64" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B64" s="35"/>
       <c r="C64" s="587" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="D64" s="329"/>
       <c r="E64" s="323"/>
@@ -26095,7 +26102,7 @@
     <row r="68" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B68" s="35"/>
       <c r="C68" s="581" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="D68" s="324"/>
       <c r="E68" s="501"/>
@@ -26112,7 +26119,7 @@
     <row r="69" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B69" s="35"/>
       <c r="C69" s="587" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="D69" s="329"/>
       <c r="E69" s="323"/>
@@ -26132,7 +26139,7 @@
     <row r="70" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B70" s="35"/>
       <c r="C70" s="587" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="D70" s="329"/>
       <c r="E70" s="323"/>
@@ -26152,7 +26159,7 @@
     <row r="71" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B71" s="35"/>
       <c r="C71" s="587" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="D71" s="329"/>
       <c r="E71" s="323"/>
@@ -26172,7 +26179,7 @@
     <row r="72" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B72" s="35"/>
       <c r="C72" s="587" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="D72" s="329"/>
       <c r="E72" s="323"/>
@@ -26192,7 +26199,7 @@
     <row r="73" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B73" s="35"/>
       <c r="C73" s="587" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="D73" s="329"/>
       <c r="E73" s="323"/>
@@ -26231,7 +26238,7 @@
     </row>
     <row r="75" spans="2:16" ht="17" x14ac:dyDescent="0.2">
       <c r="B75" s="35" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="D75" s="324"/>
       <c r="E75" s="501"/>
@@ -26256,7 +26263,7 @@
     <row r="76" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B76" s="35"/>
       <c r="C76" s="581" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="D76" s="324"/>
       <c r="E76" s="501"/>
@@ -26450,9 +26457,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B86" s="521" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="C86" s="4"/>
       <c r="D86" s="576"/>
@@ -26478,10 +26485,10 @@
     <row r="87" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B87" s="35"/>
       <c r="C87" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="D87" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E87" s="321"/>
       <c r="F87" s="337"/>
@@ -26493,7 +26500,7 @@
       <c r="M87" s="579"/>
       <c r="N87"/>
       <c r="O87" s="373" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="P87" s="370"/>
     </row>
@@ -26516,7 +26523,7 @@
     <row r="89" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B89" s="35"/>
       <c r="C89" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="D89" s="580"/>
       <c r="E89" s="562"/>
@@ -26534,10 +26541,10 @@
     <row r="90" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B90" s="35"/>
       <c r="C90" s="587" t="s">
-        <v>840</v>
+        <v>835</v>
       </c>
       <c r="D90" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E90" s="561"/>
       <c r="F90" s="337"/>
@@ -26549,17 +26556,17 @@
       <c r="M90" s="500"/>
       <c r="N90" s="67"/>
       <c r="O90" s="523" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="P90" s="370"/>
     </row>
     <row r="91" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B91" s="35"/>
       <c r="C91" s="587" t="s">
-        <v>841</v>
+        <v>836</v>
       </c>
       <c r="D91" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E91" s="561"/>
       <c r="F91" s="337"/>
@@ -26571,17 +26578,17 @@
       <c r="M91" s="500"/>
       <c r="N91" s="67"/>
       <c r="O91" s="523" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="P91" s="7"/>
     </row>
     <row r="92" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B92" s="35"/>
       <c r="C92" s="587" t="s">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="D92" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E92" s="561"/>
       <c r="F92" s="337"/>
@@ -26593,17 +26600,17 @@
       <c r="M92" s="500"/>
       <c r="N92" s="67"/>
       <c r="O92" s="523" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="P92" s="7"/>
     </row>
     <row r="93" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B93" s="35"/>
       <c r="C93" s="587" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="D93" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E93" s="561"/>
       <c r="F93" s="337"/>
@@ -26615,17 +26622,17 @@
       <c r="M93" s="500"/>
       <c r="N93" s="67"/>
       <c r="O93" s="523" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="P93" s="7"/>
     </row>
     <row r="94" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B94" s="35"/>
       <c r="C94" s="587" t="s">
-        <v>844</v>
+        <v>839</v>
       </c>
       <c r="D94" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E94" s="561"/>
       <c r="F94" s="337"/>
@@ -26637,17 +26644,17 @@
       <c r="M94" s="500"/>
       <c r="N94" s="67"/>
       <c r="O94" s="523" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="P94" s="7"/>
     </row>
     <row r="95" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B95" s="35"/>
       <c r="C95" s="587" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="D95" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E95" s="561"/>
       <c r="F95" s="337"/>
@@ -26659,17 +26666,17 @@
       <c r="M95" s="500"/>
       <c r="N95" s="67"/>
       <c r="O95" s="523" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="P95" s="370"/>
     </row>
     <row r="96" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B96" s="35"/>
       <c r="C96" s="587" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="D96" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E96" s="561"/>
       <c r="F96" s="337"/>
@@ -26681,17 +26688,17 @@
       <c r="M96" s="500"/>
       <c r="N96" s="67"/>
       <c r="O96" s="523" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="P96" s="7"/>
     </row>
     <row r="97" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B97" s="35"/>
       <c r="C97" s="587" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="D97" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E97" s="561"/>
       <c r="F97" s="337"/>
@@ -26703,17 +26710,17 @@
       <c r="M97" s="500"/>
       <c r="N97" s="67"/>
       <c r="O97" s="523" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="P97" s="7"/>
     </row>
     <row r="98" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B98" s="35"/>
       <c r="C98" s="587" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="D98" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E98" s="561"/>
       <c r="F98" s="337"/>
@@ -26725,17 +26732,17 @@
       <c r="M98" s="500"/>
       <c r="N98" s="67"/>
       <c r="O98" s="523" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="P98" s="7"/>
     </row>
     <row r="99" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B99" s="35"/>
       <c r="C99" s="587" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="D99" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E99" s="561"/>
       <c r="F99" s="337"/>
@@ -26747,17 +26754,17 @@
       <c r="M99" s="500"/>
       <c r="N99" s="67"/>
       <c r="O99" s="523" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="P99" s="7"/>
     </row>
     <row r="100" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B100" s="35"/>
       <c r="C100" s="587" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="D100" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E100" s="561"/>
       <c r="F100" s="337"/>
@@ -26769,17 +26776,17 @@
       <c r="M100" s="500"/>
       <c r="N100" s="67"/>
       <c r="O100" s="523" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="P100" s="370"/>
     </row>
     <row r="101" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B101" s="35"/>
       <c r="C101" s="587" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="D101" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E101" s="561"/>
       <c r="F101" s="337"/>
@@ -26791,17 +26798,17 @@
       <c r="M101" s="500"/>
       <c r="N101" s="67"/>
       <c r="O101" s="523" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
       <c r="P101" s="7"/>
     </row>
     <row r="102" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B102" s="35"/>
       <c r="C102" s="587" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="D102" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E102" s="561"/>
       <c r="F102" s="337"/>
@@ -26813,17 +26820,17 @@
       <c r="M102" s="500"/>
       <c r="N102" s="67"/>
       <c r="O102" s="523" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
       <c r="P102" s="7"/>
     </row>
     <row r="103" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B103" s="35"/>
       <c r="C103" s="587" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="D103" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E103" s="561"/>
       <c r="F103" s="337"/>
@@ -26835,17 +26842,17 @@
       <c r="M103" s="500"/>
       <c r="N103" s="67"/>
       <c r="O103" s="523" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="P103" s="7"/>
     </row>
     <row r="104" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B104" s="35"/>
       <c r="C104" s="587" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="D104" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E104" s="561"/>
       <c r="F104" s="337"/>
@@ -26857,17 +26864,17 @@
       <c r="M104" s="500"/>
       <c r="N104" s="67"/>
       <c r="O104" s="523" t="s">
-        <v>826</v>
+        <v>821</v>
       </c>
       <c r="P104" s="7"/>
     </row>
     <row r="105" spans="2:16" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B105" s="35"/>
       <c r="C105" s="587" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="D105" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E105" s="561"/>
       <c r="F105" s="337"/>
@@ -26879,17 +26886,17 @@
       <c r="M105" s="500"/>
       <c r="N105" s="67"/>
       <c r="O105" s="523" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="P105" s="370"/>
     </row>
     <row r="106" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B106" s="35"/>
       <c r="C106" s="587" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="D106" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E106" s="561"/>
       <c r="F106" s="337"/>
@@ -26901,17 +26908,17 @@
       <c r="M106" s="500"/>
       <c r="N106" s="67"/>
       <c r="O106" s="523" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="P106" s="7"/>
     </row>
     <row r="107" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B107" s="35"/>
       <c r="C107" s="587" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="D107" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E107" s="561"/>
       <c r="F107" s="337"/>
@@ -26923,17 +26930,17 @@
       <c r="M107" s="500"/>
       <c r="N107" s="67"/>
       <c r="O107" s="523" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
       <c r="P107" s="7"/>
     </row>
     <row r="108" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B108" s="35"/>
       <c r="C108" s="587" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="D108" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E108" s="561"/>
       <c r="F108" s="337"/>
@@ -26945,17 +26952,17 @@
       <c r="M108" s="500"/>
       <c r="N108" s="67"/>
       <c r="O108" s="523" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="P108" s="7"/>
     </row>
     <row r="109" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B109" s="35"/>
       <c r="C109" s="587" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="D109" s="580" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="E109" s="561"/>
       <c r="F109" s="337"/>
@@ -26967,7 +26974,7 @@
       <c r="M109" s="500"/>
       <c r="N109" s="67"/>
       <c r="O109" s="523" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="P109" s="7"/>
     </row>
@@ -26992,7 +26999,7 @@
     </row>
     <row r="111" spans="2:16" ht="17" x14ac:dyDescent="0.2">
       <c r="B111" s="521" t="s">
-        <v>838</v>
+        <v>833</v>
       </c>
       <c r="C111" s="4"/>
       <c r="D111" s="205"/>
@@ -27020,7 +27027,7 @@
     <row r="112" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B112" s="35"/>
       <c r="C112" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="D112" s="580"/>
       <c r="E112" s="562"/>
@@ -27038,10 +27045,10 @@
     <row r="113" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B113" s="35"/>
       <c r="C113" s="587" t="s">
-        <v>840</v>
+        <v>835</v>
       </c>
       <c r="D113" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E113" s="323"/>
       <c r="F113" s="337"/>
@@ -27053,17 +27060,17 @@
       <c r="M113" s="500"/>
       <c r="N113" s="67"/>
       <c r="O113" s="523" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="P113" s="370"/>
     </row>
     <row r="114" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B114" s="35"/>
       <c r="C114" s="587" t="s">
-        <v>841</v>
+        <v>836</v>
       </c>
       <c r="D114" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E114" s="323"/>
       <c r="F114" s="337"/>
@@ -27075,17 +27082,17 @@
       <c r="M114" s="500"/>
       <c r="N114" s="67"/>
       <c r="O114" s="523" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="P114" s="7"/>
     </row>
     <row r="115" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B115" s="35"/>
       <c r="C115" s="587" t="s">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="D115" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E115" s="323"/>
       <c r="F115" s="337"/>
@@ -27097,17 +27104,17 @@
       <c r="M115" s="500"/>
       <c r="N115" s="67"/>
       <c r="O115" s="523" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="P115" s="7"/>
     </row>
     <row r="116" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B116" s="35"/>
       <c r="C116" s="587" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="D116" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E116" s="323"/>
       <c r="F116" s="337"/>
@@ -27119,17 +27126,17 @@
       <c r="M116" s="500"/>
       <c r="N116" s="67"/>
       <c r="O116" s="523" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
       <c r="P116" s="7"/>
     </row>
     <row r="117" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B117" s="35"/>
       <c r="C117" s="587" t="s">
-        <v>844</v>
+        <v>839</v>
       </c>
       <c r="D117" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E117" s="323"/>
       <c r="F117" s="337"/>
@@ -27141,17 +27148,17 @@
       <c r="M117" s="500"/>
       <c r="N117" s="67"/>
       <c r="O117" s="523" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="P117" s="7"/>
     </row>
     <row r="118" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B118" s="35"/>
       <c r="C118" s="587" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="D118" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E118" s="323"/>
       <c r="F118" s="337"/>
@@ -27163,17 +27170,17 @@
       <c r="M118" s="500"/>
       <c r="N118" s="67"/>
       <c r="O118" s="523" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="P118" s="7"/>
     </row>
     <row r="119" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B119" s="35"/>
       <c r="C119" s="587" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="D119" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E119" s="323"/>
       <c r="F119" s="337"/>
@@ -27185,17 +27192,17 @@
       <c r="M119" s="500"/>
       <c r="N119" s="67"/>
       <c r="O119" s="523" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
       <c r="P119" s="370"/>
     </row>
     <row r="120" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B120" s="35"/>
       <c r="C120" s="587" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="D120" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E120" s="323"/>
       <c r="F120" s="337"/>
@@ -27207,17 +27214,17 @@
       <c r="M120" s="500"/>
       <c r="N120" s="67"/>
       <c r="O120" s="523" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="P120" s="7"/>
     </row>
     <row r="121" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B121" s="35"/>
       <c r="C121" s="587" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="D121" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E121" s="323"/>
       <c r="F121" s="337"/>
@@ -27229,17 +27236,17 @@
       <c r="M121" s="500"/>
       <c r="N121" s="67"/>
       <c r="O121" s="523" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="P121" s="7"/>
     </row>
     <row r="122" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B122" s="35"/>
       <c r="C122" s="587" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="D122" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E122" s="323"/>
       <c r="F122" s="337"/>
@@ -27251,17 +27258,17 @@
       <c r="M122" s="500"/>
       <c r="N122" s="67"/>
       <c r="O122" s="523" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="P122" s="7"/>
     </row>
     <row r="123" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B123" s="35"/>
       <c r="C123" s="587" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="D123" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E123" s="323"/>
       <c r="F123" s="337"/>
@@ -27273,17 +27280,17 @@
       <c r="M123" s="500"/>
       <c r="N123" s="67"/>
       <c r="O123" s="523" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="P123" s="7"/>
     </row>
     <row r="124" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B124" s="35"/>
       <c r="C124" s="587" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="D124" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E124" s="323"/>
       <c r="F124" s="337"/>
@@ -27295,17 +27302,17 @@
       <c r="M124" s="500"/>
       <c r="N124" s="67"/>
       <c r="O124" s="523" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="P124" s="7"/>
     </row>
     <row r="125" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B125" s="35"/>
       <c r="C125" s="587" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="D125" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E125" s="323"/>
       <c r="F125" s="337"/>
@@ -27317,17 +27324,17 @@
       <c r="M125" s="500"/>
       <c r="N125" s="67"/>
       <c r="O125" s="523" t="s">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="P125" s="370"/>
     </row>
     <row r="126" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B126" s="35"/>
       <c r="C126" s="587" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="D126" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E126" s="323"/>
       <c r="F126" s="337"/>
@@ -27339,17 +27346,17 @@
       <c r="M126" s="500"/>
       <c r="N126" s="67"/>
       <c r="O126" s="523" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="P126" s="7"/>
     </row>
     <row r="127" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B127" s="35"/>
       <c r="C127" s="587" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="D127" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E127" s="323"/>
       <c r="F127" s="337"/>
@@ -27361,17 +27368,17 @@
       <c r="M127" s="500"/>
       <c r="N127" s="67"/>
       <c r="O127" s="523" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="P127" s="7"/>
     </row>
     <row r="128" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B128" s="35"/>
       <c r="C128" s="587" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="D128" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E128" s="323"/>
       <c r="F128" s="337"/>
@@ -27383,17 +27390,17 @@
       <c r="M128" s="500"/>
       <c r="N128" s="67"/>
       <c r="O128" s="523" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="P128" s="7"/>
     </row>
     <row r="129" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B129" s="35"/>
       <c r="C129" s="587" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="D129" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E129" s="323"/>
       <c r="F129" s="337"/>
@@ -27405,17 +27412,17 @@
       <c r="M129" s="500"/>
       <c r="N129" s="67"/>
       <c r="O129" s="523" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="P129" s="7"/>
     </row>
     <row r="130" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B130" s="35"/>
       <c r="C130" s="587" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="D130" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E130" s="323"/>
       <c r="F130" s="337"/>
@@ -27427,17 +27434,17 @@
       <c r="M130" s="500"/>
       <c r="N130" s="67"/>
       <c r="O130" s="523" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="P130" s="7"/>
     </row>
     <row r="131" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B131" s="35"/>
       <c r="C131" s="587" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="D131" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E131" s="323"/>
       <c r="F131" s="337"/>
@@ -27449,17 +27456,17 @@
       <c r="M131" s="500"/>
       <c r="N131" s="67"/>
       <c r="O131" s="523" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="P131" s="370"/>
     </row>
     <row r="132" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B132" s="35"/>
       <c r="C132" s="587" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="D132" s="580" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="E132" s="323"/>
       <c r="F132" s="337"/>
@@ -27471,7 +27478,7 @@
       <c r="M132" s="500"/>
       <c r="N132" s="67"/>
       <c r="O132" s="523" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="P132" s="7"/>
     </row>
@@ -27738,13 +27745,13 @@
       <c r="H4" s="5"/>
     </row>
     <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="598"/>
-      <c r="C5" s="599"/>
-      <c r="D5" s="599"/>
-      <c r="E5" s="599"/>
-      <c r="F5" s="599"/>
-      <c r="G5" s="599"/>
-      <c r="H5" s="600"/>
+      <c r="B5" s="600"/>
+      <c r="C5" s="601"/>
+      <c r="D5" s="601"/>
+      <c r="E5" s="601"/>
+      <c r="F5" s="601"/>
+      <c r="G5" s="601"/>
+      <c r="H5" s="602"/>
     </row>
     <row r="6" spans="2:67" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
@@ -34583,7 +34590,7 @@
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B5" s="472" t="s">
-        <v>695</v>
+        <v>932</v>
       </c>
       <c r="C5" s="473"/>
       <c r="D5" s="473"/>
@@ -34609,10 +34616,10 @@
       <c r="C7" s="464"/>
       <c r="D7" s="464"/>
       <c r="E7" s="484" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="F7" s="457" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="G7" s="457"/>
       <c r="H7" s="456"/>
@@ -34620,7 +34627,7 @@
       <c r="J7" s="457"/>
       <c r="K7" s="476"/>
       <c r="L7" s="524" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="M7" s="524"/>
       <c r="N7" s="479"/>
@@ -34643,25 +34650,25 @@
         <v>656</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>660</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>657</v>
       </c>
       <c r="K8" s="477" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="L8" s="528" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="M8" s="528" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="N8" s="481" t="s">
         <v>639</v>
@@ -34673,7 +34680,7 @@
         <v>478</v>
       </c>
       <c r="Q8" s="482" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="R8" s="483" t="s">
         <v>641</v>
@@ -34691,19 +34698,19 @@
         <v>658</v>
       </c>
       <c r="G9" s="458" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="H9" s="458" t="s">
         <v>659</v>
       </c>
       <c r="I9" s="458" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="J9" s="458" t="s">
         <v>655</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="L9" s="525"/>
       <c r="M9" s="525"/>
@@ -34794,7 +34801,7 @@
       </c>
       <c r="D13"/>
       <c r="E13" s="16" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="F13" s="465"/>
       <c r="G13" s="465"/>
@@ -34826,7 +34833,7 @@
       </c>
       <c r="D14"/>
       <c r="E14" s="16" t="s">
-        <v>663</v>
+        <v>253</v>
       </c>
       <c r="F14" s="465"/>
       <c r="G14" s="465"/>
@@ -34858,7 +34865,7 @@
       </c>
       <c r="D15"/>
       <c r="E15" s="16" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="F15" s="465"/>
       <c r="G15" s="465"/>
@@ -34890,7 +34897,7 @@
       </c>
       <c r="D16"/>
       <c r="E16" s="16" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="F16" s="465"/>
       <c r="G16" s="465"/>
@@ -34922,7 +34929,7 @@
       </c>
       <c r="D17"/>
       <c r="E17" s="16" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="F17" s="465"/>
       <c r="G17" s="465"/>
@@ -34954,7 +34961,7 @@
       </c>
       <c r="D18"/>
       <c r="E18" s="16" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F18" s="465"/>
       <c r="G18" s="465"/>
@@ -34986,7 +34993,7 @@
       </c>
       <c r="D19"/>
       <c r="E19" s="16" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F19" s="465"/>
       <c r="G19" s="465"/>
@@ -35014,11 +35021,11 @@
     <row r="20" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B20" s="62"/>
       <c r="C20" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="D20"/>
       <c r="E20" s="16" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="F20" s="465"/>
       <c r="G20" s="465"/>
@@ -35027,30 +35034,30 @@
       <c r="J20" s="465"/>
       <c r="K20" s="486"/>
       <c r="L20" s="526">
-        <v>0.18056857232115001</v>
+        <v>0.22611100000000001</v>
       </c>
       <c r="M20" s="526">
-        <v>0.18744142455482701</v>
+        <v>0.20860999999999999</v>
       </c>
       <c r="N20" s="184"/>
       <c r="O20" s="166">
         <f>(1-M20)/L20</f>
-        <v>4.4999999999999885</v>
+        <v>3.5000066339098939</v>
       </c>
       <c r="P20"/>
       <c r="Q20"/>
       <c r="R20" s="190">
         <f>O20</f>
-        <v>4.4999999999999885</v>
+        <v>3.5000066339098939</v>
       </c>
       <c r="S20" s="215" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B21" s="62"/>
       <c r="C21" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="D21"/>
       <c r="E21" s="16"/>
@@ -35064,11 +35071,11 @@
       </c>
       <c r="H21" s="465">
         <f>L20</f>
-        <v>0.18056857232115001</v>
+        <v>0.22611100000000001</v>
       </c>
       <c r="I21" s="465">
         <f>M20</f>
-        <v>0.18744142455482701</v>
+        <v>0.20860999999999999</v>
       </c>
       <c r="J21" s="465">
         <f t="shared" si="0"/>
@@ -35095,7 +35102,7 @@
         <v>0</v>
       </c>
       <c r="S21" s="215" t="s">
-        <v>762</v>
+        <v>757</v>
       </c>
     </row>
     <row r="22" spans="2:19" x14ac:dyDescent="0.2">
@@ -35143,7 +35150,7 @@
       </c>
       <c r="D24"/>
       <c r="E24" s="16" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F24" s="465"/>
       <c r="G24" s="465"/>
@@ -35175,7 +35182,7 @@
       </c>
       <c r="D25"/>
       <c r="E25" s="16" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F25" s="465"/>
       <c r="G25" s="465"/>
@@ -35207,7 +35214,7 @@
       </c>
       <c r="D26"/>
       <c r="E26" s="16" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="F26" s="465"/>
       <c r="G26" s="465"/>
@@ -35239,7 +35246,7 @@
       </c>
       <c r="D27"/>
       <c r="E27" s="16" t="s">
-        <v>671</v>
+        <v>257</v>
       </c>
       <c r="F27" s="465"/>
       <c r="G27" s="465"/>
@@ -35271,7 +35278,7 @@
       </c>
       <c r="D28"/>
       <c r="E28" s="16" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="F28" s="465"/>
       <c r="G28" s="465"/>
@@ -35303,7 +35310,7 @@
       </c>
       <c r="D29"/>
       <c r="E29" s="16" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="F29" s="465"/>
       <c r="G29" s="465"/>
@@ -35335,7 +35342,7 @@
       </c>
       <c r="D30"/>
       <c r="E30" s="16" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="F30" s="465"/>
       <c r="G30" s="465"/>
@@ -35367,7 +35374,7 @@
       </c>
       <c r="D31"/>
       <c r="E31" s="16" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="F31" s="465"/>
       <c r="G31" s="465"/>
@@ -35399,7 +35406,7 @@
       </c>
       <c r="D32"/>
       <c r="E32" s="16" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="F32" s="465"/>
       <c r="G32" s="465"/>
@@ -35427,7 +35434,7 @@
     <row r="33" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B33" s="62"/>
       <c r="C33" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="D33"/>
       <c r="E33" s="16" t="s">
@@ -35440,30 +35447,29 @@
       <c r="J33" s="465"/>
       <c r="K33" s="486"/>
       <c r="L33" s="526">
-        <v>0.22222222222222199</v>
+        <v>0</v>
       </c>
       <c r="M33" s="526">
-        <v>0.33333333333333298</v>
+        <v>1</v>
       </c>
       <c r="N33" s="184"/>
-      <c r="O33" s="166">
-        <f>(1-M33)/L33</f>
-        <v>3.0000000000000044</v>
+      <c r="O33" s="595">
+        <v>1</v>
       </c>
       <c r="P33" s="408"/>
       <c r="Q33" s="408"/>
       <c r="R33" s="190">
         <f>O33</f>
-        <v>3.0000000000000044</v>
+        <v>1</v>
       </c>
       <c r="S33" s="215" t="s">
-        <v>763</v>
+        <v>758</v>
       </c>
     </row>
     <row r="34" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B34" s="62"/>
       <c r="C34" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="D34"/>
       <c r="E34" s="16"/>
@@ -35477,11 +35483,11 @@
       </c>
       <c r="H34" s="465">
         <f>L33</f>
-        <v>0.22222222222222199</v>
+        <v>0</v>
       </c>
       <c r="I34" s="465">
         <f>M33</f>
-        <v>0.33333333333333298</v>
+        <v>1</v>
       </c>
       <c r="J34" s="465">
         <f t="shared" si="3"/>
@@ -35499,16 +35505,16 @@
       </c>
       <c r="O34" s="166"/>
       <c r="P34"/>
-      <c r="Q34" s="465">
+      <c r="Q34" s="465" t="e">
         <f>G34*I34/((G34*I34)+((1-(SUM(H34:I34))+H34)))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="R34" s="190">
         <f>N34</f>
         <v>0</v>
       </c>
       <c r="S34" s="215" t="s">
-        <v>764</v>
+        <v>759</v>
       </c>
     </row>
     <row r="35" spans="2:19" x14ac:dyDescent="0.2">
@@ -35556,7 +35562,7 @@
       </c>
       <c r="D37"/>
       <c r="E37" s="16" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="F37" s="465"/>
       <c r="G37" s="465"/>
@@ -35588,7 +35594,7 @@
       </c>
       <c r="D38"/>
       <c r="E38" s="16" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="F38" s="465"/>
       <c r="G38" s="465"/>
@@ -35620,7 +35626,7 @@
       </c>
       <c r="D39"/>
       <c r="E39" s="16" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="F39" s="465"/>
       <c r="G39" s="465"/>
@@ -35690,7 +35696,7 @@
       </c>
       <c r="D42"/>
       <c r="E42" s="16" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="F42" s="465"/>
       <c r="G42" s="465"/>
@@ -35722,7 +35728,7 @@
       </c>
       <c r="D43"/>
       <c r="E43" s="16" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="F43" s="465"/>
       <c r="G43" s="465"/>
@@ -35754,7 +35760,7 @@
       </c>
       <c r="D44"/>
       <c r="E44" s="16" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="F44" s="465"/>
       <c r="G44" s="465"/>
@@ -35786,7 +35792,7 @@
       </c>
       <c r="D45"/>
       <c r="E45" s="16" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="F45" s="465"/>
       <c r="G45" s="465"/>
@@ -35818,7 +35824,7 @@
       </c>
       <c r="D46"/>
       <c r="E46" s="16" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="F46" s="465"/>
       <c r="G46" s="465"/>
@@ -35888,7 +35894,7 @@
       </c>
       <c r="D49"/>
       <c r="E49" s="16" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="F49" s="465"/>
       <c r="G49" s="465"/>
@@ -35917,7 +35923,7 @@
       </c>
       <c r="D50"/>
       <c r="E50" s="16" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="F50" s="465"/>
       <c r="G50" s="465"/>
@@ -35946,7 +35952,7 @@
       </c>
       <c r="D51"/>
       <c r="E51" s="16" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="F51" s="465"/>
       <c r="G51" s="465"/>

</xml_diff>